<commit_message>
feat: optimize ID Card print layout and update HRDocuments
</commit_message>
<xml_diff>
--- a/Master_Projects_2026.xlsx
+++ b/Master_Projects_2026.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X32"/>
+  <dimension ref="A1:X35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3901,30 +3901,354 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="n"/>
-      <c r="B32" s="10" t="n"/>
-      <c r="C32" s="14" t="n"/>
-      <c r="D32" s="12" t="n"/>
-      <c r="E32" s="12" t="n"/>
-      <c r="F32" s="14" t="n"/>
-      <c r="G32" s="10" t="n"/>
-      <c r="H32" s="10" t="n"/>
-      <c r="I32" s="10" t="n"/>
-      <c r="J32" s="12" t="n"/>
-      <c r="K32" s="12" t="n"/>
-      <c r="L32" s="12" t="n"/>
-      <c r="M32" s="12" t="n"/>
-      <c r="N32" s="12" t="n"/>
-      <c r="O32" s="10" t="n"/>
-      <c r="P32" s="12" t="n"/>
-      <c r="Q32" s="10" t="n"/>
-      <c r="R32" s="12" t="n"/>
-      <c r="S32" s="14" t="n"/>
-      <c r="T32" s="14" t="n"/>
-      <c r="U32" s="14" t="n"/>
-      <c r="V32" s="10" t="n"/>
-      <c r="W32" s="12" t="n"/>
-      <c r="X32" s="12" t="n"/>
+      <c r="A32" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>C5264</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="n">
+        <v>14850</v>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>BAJAJ</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>NO IDEA</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J32" s="12" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="K32" s="12" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="L32" s="12" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="M32" s="12" t="inlineStr">
+        <is>
+          <t>Gaurav Sir</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr">
+        <is>
+          <t>NO IDEA</t>
+        </is>
+      </c>
+      <c r="O32" s="10" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="P32" s="12" t="inlineStr"/>
+      <c r="Q32" s="10" t="inlineStr"/>
+      <c r="R32" s="12" t="inlineStr"/>
+      <c r="S32" s="14" t="inlineStr"/>
+      <c r="T32" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U32" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="V32" s="10" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="W32" s="12" t="inlineStr"/>
+      <c r="X32" s="12" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>C5264</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>271904</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>BAJAJ</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>NO IDEA</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>78</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Gaurav Sir</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>NO IDEA</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="T33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U33" t="n">
+        <v>78</v>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>C5292</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>34600</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>AeboCode</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>NO IDEA</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>25</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Gaurav Sir</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>NO IDEA</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="T34" t="n">
+        <v>0</v>
+      </c>
+      <c r="U34" t="n">
+        <v>25</v>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>C5295</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>42432</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>HC ROBOTICS</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>NO IDEA</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>4</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Devanshu</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Devanshu</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Devanshu</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Gaurav Sir</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comingsoon today </t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>NOIDA -&gt; ENGLABS -&gt; Hoshiarpur</t>
+        </is>
+      </c>
+      <c r="S35" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" t="n">
+        <v>4</v>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>Under Process</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr"/>
+      <c r="X35" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>